<commit_message>
Continued on working on cleaning data
</commit_message>
<xml_diff>
--- a/Pandas/Datasets/signup.xlsx
+++ b/Pandas/Datasets/signup.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/18635a36e5760d4c/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/18635a36e5760d4c/Documents/Python Data Analyses/Pandas/Datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E3D415C-4358-4A1B-B0BA-C8D28D901BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{3E3D415C-4358-4A1B-B0BA-C8D28D901BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C96FA9A3-42F2-4F1F-AB2E-09113CDEE518}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E049F67C-29B8-422E-94FA-E0897357EB19}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
   <si>
     <t>name</t>
   </si>
@@ -66,6 +66,12 @@
   </si>
   <si>
     <t>b@gmail.com</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>j@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -130,6 +136,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -449,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A69D7A4-1A2D-48DA-8774-DDA4EE96F9C6}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="18.140625" customWidth="1"/>
@@ -491,6 +501,9 @@
       <c r="C3" t="s">
         <v>8</v>
       </c>
+      <c r="D3" s="2">
+        <v>45294</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -511,9 +524,50 @@
         <v>45297</v>
       </c>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2">
+        <v>45299</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>29</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2">
+        <v>45293</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9">
+        <v>41</v>
+      </c>
+      <c r="D9" s="2">
+        <v>45296</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{F188F42D-E4DD-41A7-9A9A-4DB6103FBD50}"/>
+    <hyperlink ref="C7" r:id="rId2" xr:uid="{D32F71E0-3289-4536-999C-B39F691054FB}"/>
+    <hyperlink ref="C8" r:id="rId3" xr:uid="{9A78CB32-4CB3-4598-92F9-F199EFA095DD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Practiced with a students file with 100 kids and cleaned it using functions
</commit_message>
<xml_diff>
--- a/Pandas/Datasets/signup.xlsx
+++ b/Pandas/Datasets/signup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/18635a36e5760d4c/Documents/Python Data Analyses/Pandas/Datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{3E3D415C-4358-4A1B-B0BA-C8D28D901BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C96FA9A3-42F2-4F1F-AB2E-09113CDEE518}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{3E3D415C-4358-4A1B-B0BA-C8D28D901BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{190A0034-C435-4892-9809-546EF7DD1E58}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E049F67C-29B8-422E-94FA-E0897357EB19}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>name</t>
   </si>
@@ -520,6 +520,9 @@
       <c r="B5">
         <v>35</v>
       </c>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="D5" s="2">
         <v>45297</v>
       </c>
@@ -568,6 +571,7 @@
     <hyperlink ref="C2" r:id="rId1" xr:uid="{F188F42D-E4DD-41A7-9A9A-4DB6103FBD50}"/>
     <hyperlink ref="C7" r:id="rId2" xr:uid="{D32F71E0-3289-4536-999C-B39F691054FB}"/>
     <hyperlink ref="C8" r:id="rId3" xr:uid="{9A78CB32-4CB3-4598-92F9-F199EFA095DD}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{ECD4706A-33F3-426C-A468-CFB19AA32180}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>